<commit_message>
fix(excel): use fontFamily instead of invalid fontName
</commit_message>
<xml_diff>
--- a/docs/samples/written/アネシス寺田町　申込書.xlsx
+++ b/docs/samples/written/アネシス寺田町　申込書.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd35f0bba0eb985b/デスクトップ/VEXUM/プラージュ様/-OCR-main/-OCR-main/docs/samples/written/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{A63D28CD-9656-49D8-AA23-8B68E425E327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47F848D5-2B47-4E17-A0C8-A8051055DC09}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{A63D28CD-9656-49D8-AA23-8B68E425E327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D4B481C-B26A-43ED-8714-A90B822D2188}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D7B9D4FA-DB95-4859-9995-F738ACF57FA8}"/>
+    <workbookView minimized="1" xWindow="4890" yWindow="3310" windowWidth="14400" windowHeight="6860" xr2:uid="{D7B9D4FA-DB95-4859-9995-F738ACF57FA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2247,7 +2247,7 @@
       <c r="J17" s="44"/>
       <c r="K17" s="45"/>
       <c r="L17" s="46">
-        <f t="shared" ref="L17:L57" si="1">SUMIFS($G$14:$J$14,G17:J17,"〇")</f>
+        <f>SUMIFS($G$14:$J$14,G17:J17,"〇")</f>
         <v>0</v>
       </c>
       <c r="M17" s="47"/>
@@ -2277,7 +2277,7 @@
       <c r="J18" s="44"/>
       <c r="K18" s="45"/>
       <c r="L18" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G18:J18,"〇")</f>
         <v>0</v>
       </c>
       <c r="M18" s="47"/>
@@ -2307,7 +2307,7 @@
       <c r="J19" s="44"/>
       <c r="K19" s="45"/>
       <c r="L19" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G19:J19,"〇")</f>
         <v>0</v>
       </c>
       <c r="M19" s="47"/>
@@ -2337,7 +2337,7 @@
       <c r="J20" s="44"/>
       <c r="K20" s="45"/>
       <c r="L20" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G20:J20,"〇")</f>
         <v>0</v>
       </c>
       <c r="M20" s="47"/>
@@ -2367,7 +2367,7 @@
       <c r="J21" s="44"/>
       <c r="K21" s="45"/>
       <c r="L21" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G21:J21,"〇")</f>
         <v>0</v>
       </c>
       <c r="M21" s="47"/>
@@ -2397,7 +2397,7 @@
       <c r="J22" s="44"/>
       <c r="K22" s="45"/>
       <c r="L22" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G22:J22,"〇")</f>
         <v>0</v>
       </c>
       <c r="M22" s="47"/>
@@ -2427,7 +2427,7 @@
       <c r="J23" s="44"/>
       <c r="K23" s="45"/>
       <c r="L23" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G23:J23,"〇")</f>
         <v>0</v>
       </c>
       <c r="M23" s="47"/>
@@ -2457,7 +2457,7 @@
       <c r="J24" s="44"/>
       <c r="K24" s="45"/>
       <c r="L24" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G24:J24,"〇")</f>
         <v>0</v>
       </c>
       <c r="M24" s="47"/>
@@ -2487,7 +2487,7 @@
       <c r="J25" s="44"/>
       <c r="K25" s="45"/>
       <c r="L25" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G25:J25,"〇")</f>
         <v>0</v>
       </c>
       <c r="M25" s="47"/>
@@ -2517,7 +2517,7 @@
       <c r="J26" s="44"/>
       <c r="K26" s="45"/>
       <c r="L26" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G26:J26,"〇")</f>
         <v>0</v>
       </c>
       <c r="M26" s="47"/>
@@ -2547,7 +2547,7 @@
       <c r="J27" s="44"/>
       <c r="K27" s="45"/>
       <c r="L27" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G27:J27,"〇")</f>
         <v>0</v>
       </c>
       <c r="M27" s="47"/>
@@ -2577,7 +2577,7 @@
       <c r="J28" s="44"/>
       <c r="K28" s="45"/>
       <c r="L28" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G28:J28,"〇")</f>
         <v>0</v>
       </c>
       <c r="M28" s="47"/>
@@ -2607,7 +2607,7 @@
       <c r="J29" s="44"/>
       <c r="K29" s="45"/>
       <c r="L29" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G29:J29,"〇")</f>
         <v>0</v>
       </c>
       <c r="M29" s="47"/>
@@ -2637,7 +2637,7 @@
       <c r="J30" s="44"/>
       <c r="K30" s="45"/>
       <c r="L30" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G30:J30,"〇")</f>
         <v>0</v>
       </c>
       <c r="M30" s="47"/>
@@ -2667,7 +2667,7 @@
       <c r="J31" s="44"/>
       <c r="K31" s="45"/>
       <c r="L31" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G31:J31,"〇")</f>
         <v>0</v>
       </c>
       <c r="M31" s="47"/>
@@ -2697,7 +2697,7 @@
       <c r="J32" s="44"/>
       <c r="K32" s="45"/>
       <c r="L32" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G32:J32,"〇")</f>
         <v>0</v>
       </c>
       <c r="M32" s="47"/>
@@ -2727,7 +2727,7 @@
       <c r="J33" s="44"/>
       <c r="K33" s="45"/>
       <c r="L33" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G33:J33,"〇")</f>
         <v>0</v>
       </c>
       <c r="M33" s="47"/>
@@ -2757,7 +2757,7 @@
       <c r="J34" s="44"/>
       <c r="K34" s="45"/>
       <c r="L34" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G34:J34,"〇")</f>
         <v>0</v>
       </c>
       <c r="M34" s="47"/>
@@ -2787,7 +2787,7 @@
       <c r="J35" s="44"/>
       <c r="K35" s="45"/>
       <c r="L35" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G35:J35,"〇")</f>
         <v>0</v>
       </c>
       <c r="M35" s="47"/>
@@ -2817,7 +2817,7 @@
       <c r="J36" s="44"/>
       <c r="K36" s="45"/>
       <c r="L36" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G36:J36,"〇")</f>
         <v>0</v>
       </c>
       <c r="M36" s="47"/>
@@ -2847,7 +2847,7 @@
       <c r="J37" s="44"/>
       <c r="K37" s="45"/>
       <c r="L37" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G37:J37,"〇")</f>
         <v>0</v>
       </c>
       <c r="M37" s="47"/>
@@ -2877,7 +2877,7 @@
       <c r="J38" s="44"/>
       <c r="K38" s="45"/>
       <c r="L38" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G38:J38,"〇")</f>
         <v>0</v>
       </c>
       <c r="M38" s="47"/>
@@ -2907,7 +2907,7 @@
       <c r="J39" s="44"/>
       <c r="K39" s="45"/>
       <c r="L39" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G39:J39,"〇")</f>
         <v>0</v>
       </c>
       <c r="M39" s="47"/>
@@ -2937,7 +2937,7 @@
       <c r="J40" s="44"/>
       <c r="K40" s="45"/>
       <c r="L40" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G40:J40,"〇")</f>
         <v>0</v>
       </c>
       <c r="M40" s="47"/>
@@ -2967,7 +2967,7 @@
       <c r="J41" s="44"/>
       <c r="K41" s="45"/>
       <c r="L41" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G41:J41,"〇")</f>
         <v>0</v>
       </c>
       <c r="M41" s="47"/>
@@ -2997,7 +2997,7 @@
       <c r="J42" s="44"/>
       <c r="K42" s="45"/>
       <c r="L42" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G42:J42,"〇")</f>
         <v>0</v>
       </c>
       <c r="M42" s="47"/>
@@ -3027,7 +3027,7 @@
       <c r="J43" s="44"/>
       <c r="K43" s="45"/>
       <c r="L43" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G43:J43,"〇")</f>
         <v>0</v>
       </c>
       <c r="M43" s="47"/>
@@ -3057,7 +3057,7 @@
       <c r="J44" s="44"/>
       <c r="K44" s="45"/>
       <c r="L44" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G44:J44,"〇")</f>
         <v>0</v>
       </c>
       <c r="M44" s="47"/>
@@ -3087,7 +3087,7 @@
       <c r="J45" s="44"/>
       <c r="K45" s="45"/>
       <c r="L45" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G45:J45,"〇")</f>
         <v>0</v>
       </c>
       <c r="M45" s="47"/>
@@ -3117,7 +3117,7 @@
       <c r="J46" s="44"/>
       <c r="K46" s="45"/>
       <c r="L46" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G46:J46,"〇")</f>
         <v>0</v>
       </c>
       <c r="M46" s="47"/>
@@ -3147,7 +3147,7 @@
       <c r="J47" s="44"/>
       <c r="K47" s="45"/>
       <c r="L47" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G47:J47,"〇")</f>
         <v>0</v>
       </c>
       <c r="M47" s="47"/>
@@ -3177,7 +3177,7 @@
       <c r="J48" s="44"/>
       <c r="K48" s="45"/>
       <c r="L48" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G48:J48,"〇")</f>
         <v>0</v>
       </c>
       <c r="M48" s="47"/>
@@ -3207,7 +3207,7 @@
       <c r="J49" s="44"/>
       <c r="K49" s="45"/>
       <c r="L49" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G49:J49,"〇")</f>
         <v>0</v>
       </c>
       <c r="M49" s="47"/>
@@ -3237,7 +3237,7 @@
       <c r="J50" s="44"/>
       <c r="K50" s="45"/>
       <c r="L50" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G50:J50,"〇")</f>
         <v>0</v>
       </c>
       <c r="M50" s="47"/>
@@ -3267,7 +3267,7 @@
       <c r="J51" s="44"/>
       <c r="K51" s="45"/>
       <c r="L51" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G51:J51,"〇")</f>
         <v>0</v>
       </c>
       <c r="M51" s="47"/>
@@ -3297,7 +3297,7 @@
       <c r="J52" s="44"/>
       <c r="K52" s="45"/>
       <c r="L52" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G52:J52,"〇")</f>
         <v>0</v>
       </c>
       <c r="M52" s="47"/>
@@ -3327,7 +3327,7 @@
       <c r="J53" s="44"/>
       <c r="K53" s="45"/>
       <c r="L53" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G53:J53,"〇")</f>
         <v>0</v>
       </c>
       <c r="M53" s="47"/>
@@ -3357,7 +3357,7 @@
       <c r="J54" s="44"/>
       <c r="K54" s="45"/>
       <c r="L54" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G54:J54,"〇")</f>
         <v>0</v>
       </c>
       <c r="M54" s="47"/>
@@ -3387,7 +3387,7 @@
       <c r="J55" s="44"/>
       <c r="K55" s="45"/>
       <c r="L55" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G55:J55,"〇")</f>
         <v>0</v>
       </c>
       <c r="M55" s="47"/>
@@ -3417,7 +3417,7 @@
       <c r="J56" s="44"/>
       <c r="K56" s="45"/>
       <c r="L56" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G56:J56,"〇")</f>
         <v>0</v>
       </c>
       <c r="M56" s="47"/>
@@ -3447,7 +3447,7 @@
       <c r="J57" s="44"/>
       <c r="K57" s="45"/>
       <c r="L57" s="46">
-        <f t="shared" si="1"/>
+        <f>SUMIFS($G$14:$J$14,G57:J57,"〇")</f>
         <v>0</v>
       </c>
       <c r="M57" s="47"/>

</xml_diff>